<commit_message>
implemented function to get unique verb infinitives
</commit_message>
<xml_diff>
--- a/verbs excel.xlsx
+++ b/verbs excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tthol\OneDrive\Bureaublad\de echte git programmaties\spanish verb conjugations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38C84A5E-B864-4968-A061-9C627DF952EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AEAFC88-4031-40C7-90B6-6F39CDB7D4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D7A2D11E-8C70-4A47-8240-C068B3A068CB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="25">
   <si>
     <t>verb</t>
   </si>
@@ -105,6 +105,15 @@
   </si>
   <si>
     <t>habláis</t>
+  </si>
+  <si>
+    <t>comer</t>
+  </si>
+  <si>
+    <t>er</t>
+  </si>
+  <si>
+    <t>como</t>
   </si>
 </sst>
 </file>
@@ -476,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B58F3D2-A6FC-480F-9E63-40051C7B64BB}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -619,6 +628,26 @@
         <v>20</v>
       </c>
     </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>